<commit_message>
forward: liquida o historico de agosto e inicio de setembro (697 jogos)
A pagina mostrava agosto com apenas 7-16% dos jogos com resultado e a 1a
quinzena de setembro com 37%. Os placares existiam nas bases (betfair oficial,
base betfair, b365, planilhas, manuais) -- faltava o cruzamento.

Regra de GREEN/RED validada antes de escrever: aplicada aos 680 jogos que ja
tinham resultado e placar numerico, reproduziu 680/680 sem divergencia.

Cobertura depois: 100% / 98,5% / 98% / 100% / 100% por quinzena. Sobraram 10
jogos sem placar em 1.622. Backups .bak_hist12out por planilha.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-01.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-01.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sinais_Aprovados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -595,12 +595,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -761,12 +761,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0x0</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -840,12 +840,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2x2</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -919,12 +919,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>1x1</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="P6" t="inlineStr"/>
@@ -998,12 +998,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>1x1</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>4x3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,12 +1156,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2x0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
@@ -1322,12 +1322,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0x1</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
@@ -1488,12 +1488,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0x4</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
@@ -1567,12 +1567,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>3x0</t>
+          <t>3-0</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
@@ -1725,12 +1725,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0x3</t>
+          <t>0-3</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>5x1</t>
+          <t>5-1</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
@@ -1883,12 +1883,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
@@ -1962,12 +1962,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P19" t="inlineStr"/>
@@ -2041,12 +2041,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0x0</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
@@ -2120,12 +2120,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>3x4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
@@ -2199,12 +2199,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>0x1</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -2278,12 +2278,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2x2</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -2357,12 +2357,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>3x2</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>1x3</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -2515,12 +2515,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>0x1</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>3x1</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>

</xml_diff>

<commit_message>
revert: desfaz o preenchimento dos 697 resultados (volta ao original)
Os 697 resultados que eu preenchi em 01/08-15/09 eram automacao em cima de
automacao -- 651 deles ja tinham placar na planilha, posto por outro script.
Nao acrescentavam registro do usuario e misturavam as origens.

46 planilhas restauradas dos backups .bak_hist12out e verificadas uma a uma:
identicas ao original, zero diferencas.

Mantidos os dois consertos de codigo, que nao tocam em dado: c7d6606 (BOM na
liquidacao do ledger) e 65d6244 (pagina 02 lendo o ledger).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-01.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-01.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sinais_Aprovados" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -595,12 +595,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -761,12 +761,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>0x0</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -840,12 +840,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>2x2</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -919,12 +919,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1x1</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P6" t="inlineStr"/>
@@ -998,12 +998,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1x1</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>RED</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4x3</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,12 +1156,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>2x0</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
@@ -1322,12 +1322,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0x1</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
@@ -1488,12 +1488,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0-4</t>
+          <t>0x4</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
@@ -1567,12 +1567,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>1x0</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>3-0</t>
+          <t>3x0</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
@@ -1725,12 +1725,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>0x3</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>5-1</t>
+          <t>5x1</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
@@ -1883,12 +1883,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>1x0</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
@@ -1962,12 +1962,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>1x0</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P19" t="inlineStr"/>
@@ -2041,12 +2041,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>0x0</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
@@ -2120,12 +2120,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3x4</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
@@ -2199,12 +2199,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0x1</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -2278,12 +2278,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>2x2</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -2357,12 +2357,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3x2</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>1x3</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -2515,12 +2515,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0x1</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2594,12 +2594,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>3x1</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>PENDENTE</t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>

</xml_diff>